<commit_message>
feat: implement new GUI for shift planning and management using CustomTkinter
</commit_message>
<xml_diff>
--- a/turnos_Septiembre_2026.xlsx
+++ b/turnos_Septiembre_2026.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,8 +59,11 @@
       <b val="1"/>
       <sz val="14"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -113,6 +116,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FF3B30"/>
         <bgColor rgb="00FF3B30"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B45309"/>
+        <bgColor rgb="00B45309"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B21B6"/>
+        <bgColor rgb="005B21B6"/>
       </patternFill>
     </fill>
   </fills>
@@ -190,7 +205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -334,9 +349,16 @@
     <xf numFmtId="49" fontId="0" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment shrinkToFit="1"/>
     </xf>
@@ -358,16 +380,12 @@
     <xf numFmtId="49" fontId="2" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="6" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="11" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1018,11 +1036,11 @@
       <c r="S4" s="46" t="n"/>
       <c r="T4" s="54" t="n"/>
       <c r="U4" s="54" t="n"/>
-      <c r="V4" s="47" t="n"/>
-      <c r="W4" s="47" t="n"/>
-      <c r="X4" s="47" t="n"/>
-      <c r="Y4" s="47" t="n"/>
-      <c r="Z4" s="47" t="n"/>
+      <c r="V4" s="55" t="n"/>
+      <c r="W4" s="55" t="n"/>
+      <c r="X4" s="55" t="n"/>
+      <c r="Y4" s="55" t="n"/>
+      <c r="Z4" s="55" t="n"/>
       <c r="AA4" s="55" t="n"/>
       <c r="AB4" s="55" t="n"/>
       <c r="AC4" s="47" t="n"/>
@@ -1056,18 +1074,18 @@
       <c r="Q5" s="46" t="n"/>
       <c r="R5" s="46" t="n"/>
       <c r="S5" s="47" t="n"/>
-      <c r="T5" s="55" t="n"/>
-      <c r="U5" s="55" t="n"/>
+      <c r="T5" s="56" t="n"/>
+      <c r="U5" s="56" t="n"/>
       <c r="V5" s="47" t="n"/>
       <c r="W5" s="47" t="n"/>
       <c r="X5" s="47" t="n"/>
       <c r="Y5" s="47" t="n"/>
       <c r="Z5" s="47" t="n"/>
-      <c r="AA5" s="55" t="n"/>
-      <c r="AB5" s="55" t="n"/>
-      <c r="AC5" s="47" t="n"/>
-      <c r="AD5" s="46" t="n"/>
-      <c r="AE5" s="19" t="n"/>
+      <c r="AA5" s="56" t="n"/>
+      <c r="AB5" s="56" t="n"/>
+      <c r="AC5" s="55" t="n"/>
+      <c r="AD5" s="57" t="n"/>
+      <c r="AE5" s="58" t="n"/>
       <c r="AF5" s="19" t="n"/>
       <c r="AG5" s="19" t="n"/>
       <c r="AH5" s="19" t="n"/>
@@ -1082,8 +1100,8 @@
       <c r="C6" s="46" t="n"/>
       <c r="D6" s="46" t="n"/>
       <c r="E6" s="46" t="n"/>
-      <c r="F6" s="55" t="n"/>
-      <c r="G6" s="55" t="n"/>
+      <c r="F6" s="56" t="n"/>
+      <c r="G6" s="56" t="n"/>
       <c r="H6" s="46" t="n"/>
       <c r="I6" s="46" t="n"/>
       <c r="J6" s="46" t="n"/>
@@ -1122,8 +1140,8 @@
       <c r="C7" s="46" t="n"/>
       <c r="D7" s="46" t="n"/>
       <c r="E7" s="46" t="n"/>
-      <c r="F7" s="55" t="n"/>
-      <c r="G7" s="55" t="n"/>
+      <c r="F7" s="56" t="n"/>
+      <c r="G7" s="56" t="n"/>
       <c r="H7" s="46" t="n"/>
       <c r="I7" s="46" t="n"/>
       <c r="J7" s="46" t="n"/>
@@ -1136,8 +1154,8 @@
       <c r="Q7" s="47" t="n"/>
       <c r="R7" s="47" t="n"/>
       <c r="S7" s="47" t="n"/>
-      <c r="T7" s="56" t="n"/>
-      <c r="U7" s="56" t="n"/>
+      <c r="T7" s="59" t="n"/>
+      <c r="U7" s="59" t="n"/>
       <c r="V7" s="46" t="n"/>
       <c r="W7" s="46" t="n"/>
       <c r="X7" s="46" t="n"/>
@@ -1162,29 +1180,29 @@
       <c r="C8" s="45" t="n"/>
       <c r="D8" s="45" t="n"/>
       <c r="E8" s="45" t="n"/>
-      <c r="F8" s="57" t="n"/>
-      <c r="G8" s="57" t="n"/>
+      <c r="F8" s="60" t="n"/>
+      <c r="G8" s="60" t="n"/>
       <c r="H8" s="45" t="n"/>
       <c r="I8" s="45" t="n"/>
       <c r="J8" s="45" t="n"/>
       <c r="K8" s="45" t="n"/>
       <c r="L8" s="45" t="n"/>
-      <c r="M8" s="58" t="n"/>
-      <c r="N8" s="58" t="n"/>
+      <c r="M8" s="61" t="n"/>
+      <c r="N8" s="61" t="n"/>
       <c r="O8" s="18" t="n"/>
       <c r="P8" s="18" t="n"/>
       <c r="Q8" s="18" t="n"/>
       <c r="R8" s="18" t="n"/>
       <c r="S8" s="18" t="n"/>
-      <c r="T8" s="59" t="n"/>
-      <c r="U8" s="59" t="n"/>
+      <c r="T8" s="62" t="n"/>
+      <c r="U8" s="62" t="n"/>
       <c r="V8" s="18" t="n"/>
       <c r="W8" s="18" t="n"/>
       <c r="X8" s="18" t="n"/>
       <c r="Y8" s="18" t="n"/>
       <c r="Z8" s="18" t="n"/>
-      <c r="AA8" s="57" t="n"/>
-      <c r="AB8" s="57" t="n"/>
+      <c r="AA8" s="60" t="n"/>
+      <c r="AB8" s="60" t="n"/>
       <c r="AC8" s="18" t="n"/>
       <c r="AD8" s="45" t="n"/>
       <c r="AE8" s="19" t="n"/>
@@ -1202,8 +1220,8 @@
       <c r="C9" s="46" t="n"/>
       <c r="D9" s="46" t="n"/>
       <c r="E9" s="46" t="n"/>
-      <c r="F9" s="55" t="n"/>
-      <c r="G9" s="55" t="n"/>
+      <c r="F9" s="56" t="n"/>
+      <c r="G9" s="56" t="n"/>
       <c r="H9" s="46" t="n"/>
       <c r="I9" s="46" t="n"/>
       <c r="J9" s="46" t="n"/>
@@ -1216,8 +1234,8 @@
       <c r="Q9" s="47" t="n"/>
       <c r="R9" s="47" t="n"/>
       <c r="S9" s="47" t="n"/>
-      <c r="T9" s="56" t="n"/>
-      <c r="U9" s="56" t="n"/>
+      <c r="T9" s="59" t="n"/>
+      <c r="U9" s="59" t="n"/>
       <c r="V9" s="46" t="n"/>
       <c r="W9" s="46" t="n"/>
       <c r="X9" s="46" t="n"/>
@@ -1242,29 +1260,29 @@
       <c r="C10" s="46" t="n"/>
       <c r="D10" s="18" t="n"/>
       <c r="E10" s="46" t="n"/>
-      <c r="F10" s="55" t="n"/>
-      <c r="G10" s="57" t="n"/>
+      <c r="F10" s="56" t="n"/>
+      <c r="G10" s="60" t="n"/>
       <c r="H10" s="46" t="n"/>
       <c r="I10" s="46" t="n"/>
       <c r="J10" s="18" t="n"/>
       <c r="K10" s="46" t="n"/>
       <c r="L10" s="46" t="n"/>
-      <c r="M10" s="57" t="n"/>
+      <c r="M10" s="60" t="n"/>
       <c r="N10" s="54" t="n"/>
       <c r="O10" s="47" t="n"/>
       <c r="P10" s="18" t="n"/>
       <c r="Q10" s="47" t="n"/>
       <c r="R10" s="47" t="n"/>
       <c r="S10" s="18" t="n"/>
-      <c r="T10" s="56" t="n"/>
-      <c r="U10" s="56" t="n"/>
+      <c r="T10" s="59" t="n"/>
+      <c r="U10" s="59" t="n"/>
       <c r="V10" s="18" t="n"/>
       <c r="W10" s="46" t="n"/>
       <c r="X10" s="46" t="n"/>
       <c r="Y10" s="46" t="n"/>
       <c r="Z10" s="46" t="n"/>
       <c r="AA10" s="54" t="n"/>
-      <c r="AB10" s="58" t="n"/>
+      <c r="AB10" s="61" t="n"/>
       <c r="AC10" s="45" t="n"/>
       <c r="AD10" s="18" t="n"/>
       <c r="AE10" s="39" t="n"/>
@@ -1282,22 +1300,22 @@
       <c r="C11" s="47" t="n"/>
       <c r="D11" s="47" t="n"/>
       <c r="E11" s="47" t="n"/>
-      <c r="F11" s="55" t="n"/>
-      <c r="G11" s="55" t="n"/>
+      <c r="F11" s="56" t="n"/>
+      <c r="G11" s="56" t="n"/>
       <c r="H11" s="46" t="n"/>
       <c r="I11" s="46" t="n"/>
       <c r="J11" s="46" t="n"/>
-      <c r="K11" s="60" t="n"/>
-      <c r="L11" s="60" t="n"/>
-      <c r="M11" s="61" t="n"/>
-      <c r="N11" s="61" t="n"/>
-      <c r="O11" s="60" t="n"/>
-      <c r="P11" s="60" t="n"/>
-      <c r="Q11" s="60" t="n"/>
+      <c r="K11" s="63" t="n"/>
+      <c r="L11" s="63" t="n"/>
+      <c r="M11" s="64" t="n"/>
+      <c r="N11" s="64" t="n"/>
+      <c r="O11" s="63" t="n"/>
+      <c r="P11" s="63" t="n"/>
+      <c r="Q11" s="63" t="n"/>
       <c r="R11" s="46" t="n"/>
       <c r="S11" s="46" t="n"/>
-      <c r="T11" s="56" t="n"/>
-      <c r="U11" s="56" t="n"/>
+      <c r="T11" s="59" t="n"/>
+      <c r="U11" s="59" t="n"/>
       <c r="V11" s="46" t="n"/>
       <c r="W11" s="46" t="n"/>
       <c r="X11" s="46" t="n"/>
@@ -1322,29 +1340,29 @@
       <c r="C12" s="46" t="n"/>
       <c r="D12" s="46" t="n"/>
       <c r="E12" s="18" t="n"/>
-      <c r="F12" s="57" t="n"/>
-      <c r="G12" s="55" t="n"/>
+      <c r="F12" s="60" t="n"/>
+      <c r="G12" s="56" t="n"/>
       <c r="H12" s="45" t="n"/>
       <c r="I12" s="45" t="n"/>
       <c r="J12" s="46" t="n"/>
       <c r="K12" s="45" t="n"/>
       <c r="L12" s="45" t="n"/>
       <c r="M12" s="54" t="n"/>
-      <c r="N12" s="58" t="n"/>
+      <c r="N12" s="61" t="n"/>
       <c r="O12" s="45" t="n"/>
       <c r="P12" s="46" t="n"/>
       <c r="Q12" s="45" t="n"/>
       <c r="R12" s="45" t="n"/>
       <c r="S12" s="46" t="n"/>
-      <c r="T12" s="58" t="n"/>
-      <c r="U12" s="58" t="n"/>
+      <c r="T12" s="61" t="n"/>
+      <c r="U12" s="61" t="n"/>
       <c r="V12" s="46" t="n"/>
       <c r="W12" s="45" t="n"/>
       <c r="X12" s="45" t="n"/>
       <c r="Y12" s="45" t="n"/>
       <c r="Z12" s="45" t="n"/>
-      <c r="AA12" s="58" t="n"/>
-      <c r="AB12" s="58" t="n"/>
+      <c r="AA12" s="61" t="n"/>
+      <c r="AB12" s="61" t="n"/>
       <c r="AC12" s="45" t="n"/>
       <c r="AD12" s="18" t="n"/>
       <c r="AE12" s="19" t="n"/>
@@ -1362,8 +1380,8 @@
       <c r="C13" s="47" t="n"/>
       <c r="D13" s="47" t="n"/>
       <c r="E13" s="47" t="n"/>
-      <c r="F13" s="55" t="n"/>
-      <c r="G13" s="55" t="n"/>
+      <c r="F13" s="56" t="n"/>
+      <c r="G13" s="56" t="n"/>
       <c r="H13" s="46" t="n"/>
       <c r="I13" s="46" t="n"/>
       <c r="J13" s="46" t="n"/>
@@ -1383,8 +1401,8 @@
       <c r="X13" s="18" t="n"/>
       <c r="Y13" s="18" t="n"/>
       <c r="Z13" s="18" t="n"/>
-      <c r="AA13" s="57" t="n"/>
-      <c r="AB13" s="57" t="n"/>
+      <c r="AA13" s="60" t="n"/>
+      <c r="AB13" s="60" t="n"/>
       <c r="AC13" s="18" t="n"/>
       <c r="AD13" s="46" t="n"/>
       <c r="AE13" s="19" t="n"/>
@@ -1402,8 +1420,8 @@
       <c r="C14" s="47" t="n"/>
       <c r="D14" s="47" t="n"/>
       <c r="E14" s="47" t="n"/>
-      <c r="F14" s="55" t="n"/>
-      <c r="G14" s="55" t="n"/>
+      <c r="F14" s="56" t="n"/>
+      <c r="G14" s="56" t="n"/>
       <c r="H14" s="46" t="n"/>
       <c r="I14" s="46" t="n"/>
       <c r="J14" s="46" t="n"/>
@@ -1423,8 +1441,8 @@
       <c r="X14" s="18" t="n"/>
       <c r="Y14" s="18" t="n"/>
       <c r="Z14" s="18" t="n"/>
-      <c r="AA14" s="57" t="n"/>
-      <c r="AB14" s="57" t="n"/>
+      <c r="AA14" s="60" t="n"/>
+      <c r="AB14" s="60" t="n"/>
       <c r="AC14" s="18" t="n"/>
       <c r="AD14" s="46" t="n"/>
       <c r="AE14" s="19" t="n"/>
@@ -1438,33 +1456,33 @@
           <t>PRO ROSAS FERNANDEZ RODRIGO</t>
         </is>
       </c>
-      <c r="B15" s="62" t="n"/>
-      <c r="C15" s="62" t="n"/>
-      <c r="D15" s="63" t="n"/>
-      <c r="E15" s="62" t="n"/>
-      <c r="F15" s="62" t="n"/>
-      <c r="G15" s="63" t="n"/>
+      <c r="B15" s="65" t="n"/>
+      <c r="C15" s="65" t="n"/>
+      <c r="D15" s="55" t="n"/>
+      <c r="E15" s="65" t="n"/>
+      <c r="F15" s="65" t="n"/>
+      <c r="G15" s="55" t="n"/>
       <c r="H15" s="45" t="n"/>
       <c r="I15" s="45" t="n"/>
       <c r="J15" s="46" t="n"/>
       <c r="K15" s="45" t="n"/>
       <c r="L15" s="45" t="n"/>
       <c r="M15" s="54" t="n"/>
-      <c r="N15" s="58" t="n"/>
+      <c r="N15" s="61" t="n"/>
       <c r="O15" s="45" t="n"/>
       <c r="P15" s="46" t="n"/>
       <c r="Q15" s="45" t="n"/>
       <c r="R15" s="45" t="n"/>
       <c r="S15" s="46" t="n"/>
-      <c r="T15" s="58" t="n"/>
-      <c r="U15" s="58" t="n"/>
+      <c r="T15" s="61" t="n"/>
+      <c r="U15" s="61" t="n"/>
       <c r="V15" s="47" t="n"/>
       <c r="W15" s="18" t="n"/>
       <c r="X15" s="18" t="n"/>
       <c r="Y15" s="18" t="n"/>
       <c r="Z15" s="18" t="n"/>
-      <c r="AA15" s="57" t="n"/>
-      <c r="AB15" s="57" t="n"/>
+      <c r="AA15" s="60" t="n"/>
+      <c r="AB15" s="60" t="n"/>
       <c r="AC15" s="18" t="n"/>
       <c r="AD15" s="46" t="n"/>
       <c r="AE15" s="19" t="n"/>
@@ -1482,29 +1500,37 @@
       <c r="C16" s="18" t="n"/>
       <c r="D16" s="47" t="n"/>
       <c r="E16" s="18" t="n"/>
-      <c r="F16" s="57" t="n"/>
-      <c r="G16" s="55" t="n"/>
-      <c r="H16" s="64" t="n"/>
-      <c r="I16" s="64" t="n"/>
-      <c r="J16" s="65" t="n"/>
-      <c r="K16" s="64" t="n"/>
-      <c r="L16" s="64" t="n"/>
-      <c r="M16" s="65" t="n"/>
-      <c r="N16" s="62" t="n"/>
+      <c r="F16" s="60" t="n"/>
+      <c r="G16" s="56" t="n"/>
+      <c r="H16" s="45" t="n"/>
+      <c r="I16" s="66" t="inlineStr">
+        <is>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="J16" s="66" t="inlineStr">
+        <is>
+          <t>DA</t>
+        </is>
+      </c>
+      <c r="K16" s="45" t="n"/>
+      <c r="L16" s="45" t="n"/>
+      <c r="M16" s="54" t="n"/>
+      <c r="N16" s="60" t="n"/>
       <c r="O16" s="18" t="n"/>
       <c r="P16" s="46" t="n"/>
       <c r="Q16" s="18" t="n"/>
       <c r="R16" s="18" t="n"/>
       <c r="S16" s="46" t="n"/>
-      <c r="T16" s="57" t="n"/>
-      <c r="U16" s="57" t="n"/>
+      <c r="T16" s="60" t="n"/>
+      <c r="U16" s="60" t="n"/>
       <c r="V16" s="46" t="n"/>
       <c r="W16" s="18" t="n"/>
       <c r="X16" s="18" t="n"/>
       <c r="Y16" s="18" t="n"/>
       <c r="Z16" s="18" t="n"/>
-      <c r="AA16" s="57" t="n"/>
-      <c r="AB16" s="57" t="n"/>
+      <c r="AA16" s="60" t="n"/>
+      <c r="AB16" s="60" t="n"/>
       <c r="AC16" s="18" t="n"/>
       <c r="AD16" s="46" t="n"/>
       <c r="AE16" s="19" t="n"/>
@@ -1522,22 +1548,22 @@
       <c r="C17" s="47" t="n"/>
       <c r="D17" s="47" t="n"/>
       <c r="E17" s="47" t="n"/>
-      <c r="F17" s="55" t="n"/>
-      <c r="G17" s="55" t="n"/>
-      <c r="H17" s="46" t="n"/>
-      <c r="I17" s="46" t="n"/>
-      <c r="J17" s="46" t="n"/>
-      <c r="K17" s="46" t="n"/>
-      <c r="L17" s="46" t="n"/>
-      <c r="M17" s="54" t="n"/>
-      <c r="N17" s="54" t="n"/>
-      <c r="O17" s="65" t="n"/>
-      <c r="P17" s="65" t="n"/>
-      <c r="Q17" s="65" t="n"/>
-      <c r="R17" s="65" t="n"/>
-      <c r="S17" s="65" t="n"/>
-      <c r="T17" s="65" t="n"/>
-      <c r="U17" s="65" t="n"/>
+      <c r="F17" s="56" t="n"/>
+      <c r="G17" s="56" t="n"/>
+      <c r="H17" s="57" t="n"/>
+      <c r="I17" s="57" t="n"/>
+      <c r="J17" s="57" t="n"/>
+      <c r="K17" s="57" t="n"/>
+      <c r="L17" s="57" t="n"/>
+      <c r="M17" s="57" t="n"/>
+      <c r="N17" s="57" t="n"/>
+      <c r="O17" s="46" t="n"/>
+      <c r="P17" s="46" t="n"/>
+      <c r="Q17" s="46" t="n"/>
+      <c r="R17" s="46" t="n"/>
+      <c r="S17" s="46" t="n"/>
+      <c r="T17" s="54" t="n"/>
+      <c r="U17" s="54" t="n"/>
       <c r="V17" s="46" t="n"/>
       <c r="W17" s="46" t="n"/>
       <c r="X17" s="46" t="n"/>
@@ -1571,20 +1597,20 @@
       <c r="L18" s="46" t="n"/>
       <c r="M18" s="54" t="n"/>
       <c r="N18" s="54" t="n"/>
-      <c r="O18" s="46" t="n"/>
-      <c r="P18" s="46" t="n"/>
-      <c r="Q18" s="46" t="n"/>
-      <c r="R18" s="46" t="n"/>
-      <c r="S18" s="46" t="n"/>
-      <c r="T18" s="54" t="n"/>
-      <c r="U18" s="54" t="n"/>
-      <c r="V18" s="65" t="n"/>
-      <c r="W18" s="65" t="n"/>
-      <c r="X18" s="65" t="n"/>
-      <c r="Y18" s="65" t="n"/>
-      <c r="Z18" s="65" t="n"/>
-      <c r="AA18" s="65" t="n"/>
-      <c r="AB18" s="65" t="n"/>
+      <c r="O18" s="57" t="n"/>
+      <c r="P18" s="57" t="n"/>
+      <c r="Q18" s="57" t="n"/>
+      <c r="R18" s="57" t="n"/>
+      <c r="S18" s="57" t="n"/>
+      <c r="T18" s="57" t="n"/>
+      <c r="U18" s="57" t="n"/>
+      <c r="V18" s="46" t="n"/>
+      <c r="W18" s="46" t="n"/>
+      <c r="X18" s="46" t="n"/>
+      <c r="Y18" s="46" t="n"/>
+      <c r="Z18" s="46" t="n"/>
+      <c r="AA18" s="54" t="n"/>
+      <c r="AB18" s="54" t="n"/>
       <c r="AC18" s="46" t="n"/>
       <c r="AD18" s="46" t="n"/>
       <c r="AE18" s="19" t="n"/>
@@ -1609,8 +1635,8 @@
       <c r="J19" s="47" t="n"/>
       <c r="K19" s="47" t="n"/>
       <c r="L19" s="47" t="n"/>
-      <c r="M19" s="55" t="n"/>
-      <c r="N19" s="55" t="n"/>
+      <c r="M19" s="56" t="n"/>
+      <c r="N19" s="56" t="n"/>
       <c r="O19" s="46" t="n"/>
       <c r="P19" s="46" t="n"/>
       <c r="Q19" s="46" t="n"/>
@@ -1619,15 +1645,27 @@
       <c r="T19" s="54" t="n"/>
       <c r="U19" s="54" t="n"/>
       <c r="V19" s="46" t="n"/>
-      <c r="W19" s="46" t="n"/>
-      <c r="X19" s="46" t="n"/>
-      <c r="Y19" s="46" t="n"/>
+      <c r="W19" s="67" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="X19" s="67" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="Y19" s="67" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
       <c r="Z19" s="46" t="n"/>
       <c r="AA19" s="54" t="n"/>
       <c r="AB19" s="54" t="n"/>
-      <c r="AC19" s="65" t="n"/>
-      <c r="AD19" s="62" t="n"/>
-      <c r="AE19" s="66" t="n"/>
+      <c r="AC19" s="46" t="n"/>
+      <c r="AD19" s="18" t="n"/>
+      <c r="AE19" s="19" t="n"/>
       <c r="AF19" s="19" t="n"/>
       <c r="AG19" s="19" t="n"/>
       <c r="AH19" s="19" t="n"/>

</xml_diff>

<commit_message>
Add new exception types and enhance Excel export functionality
- Introduced new exception types: Licencia (LIC) and Otros (OTR) with corresponding colors in the GUI.
- Updated the ExcelHandler to apply new fill patterns for the added exception types.
- Modified the TurnosApp to include radio buttons for selecting the new exception types.
- Enhanced the save and export functionality to allow saving the current month and exporting to Excel.
- Updated UI texts for clarity and consistency.
- Added a new button for exporting the calendar to Excel.
- Refactored code to improve readability and maintainability.
</commit_message>
<xml_diff>
--- a/turnos_Septiembre_2026.xlsx
+++ b/turnos_Septiembre_2026.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,11 +59,8 @@
       <b val="1"/>
       <sz val="14"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
-  <fills count="12">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -116,18 +113,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FF3B30"/>
         <bgColor rgb="00FF3B30"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00B45309"/>
-        <bgColor rgb="00B45309"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="005B21B6"/>
-        <bgColor rgb="005B21B6"/>
       </patternFill>
     </fill>
   </fills>
@@ -205,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -349,16 +334,9 @@
     <xf numFmtId="49" fontId="0" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment shrinkToFit="1"/>
     </xf>
@@ -380,12 +358,16 @@
     <xf numFmtId="49" fontId="2" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="11" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="49" fontId="2" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1036,11 +1018,11 @@
       <c r="S4" s="46" t="n"/>
       <c r="T4" s="54" t="n"/>
       <c r="U4" s="54" t="n"/>
-      <c r="V4" s="55" t="n"/>
-      <c r="W4" s="55" t="n"/>
-      <c r="X4" s="55" t="n"/>
-      <c r="Y4" s="55" t="n"/>
-      <c r="Z4" s="55" t="n"/>
+      <c r="V4" s="47" t="n"/>
+      <c r="W4" s="47" t="n"/>
+      <c r="X4" s="47" t="n"/>
+      <c r="Y4" s="47" t="n"/>
+      <c r="Z4" s="47" t="n"/>
       <c r="AA4" s="55" t="n"/>
       <c r="AB4" s="55" t="n"/>
       <c r="AC4" s="47" t="n"/>
@@ -1074,18 +1056,18 @@
       <c r="Q5" s="46" t="n"/>
       <c r="R5" s="46" t="n"/>
       <c r="S5" s="47" t="n"/>
-      <c r="T5" s="56" t="n"/>
-      <c r="U5" s="56" t="n"/>
+      <c r="T5" s="55" t="n"/>
+      <c r="U5" s="55" t="n"/>
       <c r="V5" s="47" t="n"/>
       <c r="W5" s="47" t="n"/>
       <c r="X5" s="47" t="n"/>
       <c r="Y5" s="47" t="n"/>
       <c r="Z5" s="47" t="n"/>
-      <c r="AA5" s="56" t="n"/>
-      <c r="AB5" s="56" t="n"/>
-      <c r="AC5" s="55" t="n"/>
-      <c r="AD5" s="57" t="n"/>
-      <c r="AE5" s="58" t="n"/>
+      <c r="AA5" s="55" t="n"/>
+      <c r="AB5" s="55" t="n"/>
+      <c r="AC5" s="47" t="n"/>
+      <c r="AD5" s="46" t="n"/>
+      <c r="AE5" s="19" t="n"/>
       <c r="AF5" s="19" t="n"/>
       <c r="AG5" s="19" t="n"/>
       <c r="AH5" s="19" t="n"/>
@@ -1100,8 +1082,8 @@
       <c r="C6" s="46" t="n"/>
       <c r="D6" s="46" t="n"/>
       <c r="E6" s="46" t="n"/>
-      <c r="F6" s="56" t="n"/>
-      <c r="G6" s="56" t="n"/>
+      <c r="F6" s="55" t="n"/>
+      <c r="G6" s="55" t="n"/>
       <c r="H6" s="46" t="n"/>
       <c r="I6" s="46" t="n"/>
       <c r="J6" s="46" t="n"/>
@@ -1140,8 +1122,8 @@
       <c r="C7" s="46" t="n"/>
       <c r="D7" s="46" t="n"/>
       <c r="E7" s="46" t="n"/>
-      <c r="F7" s="56" t="n"/>
-      <c r="G7" s="56" t="n"/>
+      <c r="F7" s="55" t="n"/>
+      <c r="G7" s="55" t="n"/>
       <c r="H7" s="46" t="n"/>
       <c r="I7" s="46" t="n"/>
       <c r="J7" s="46" t="n"/>
@@ -1154,8 +1136,8 @@
       <c r="Q7" s="47" t="n"/>
       <c r="R7" s="47" t="n"/>
       <c r="S7" s="47" t="n"/>
-      <c r="T7" s="59" t="n"/>
-      <c r="U7" s="59" t="n"/>
+      <c r="T7" s="56" t="n"/>
+      <c r="U7" s="56" t="n"/>
       <c r="V7" s="46" t="n"/>
       <c r="W7" s="46" t="n"/>
       <c r="X7" s="46" t="n"/>
@@ -1180,29 +1162,29 @@
       <c r="C8" s="45" t="n"/>
       <c r="D8" s="45" t="n"/>
       <c r="E8" s="45" t="n"/>
-      <c r="F8" s="60" t="n"/>
-      <c r="G8" s="60" t="n"/>
+      <c r="F8" s="57" t="n"/>
+      <c r="G8" s="57" t="n"/>
       <c r="H8" s="45" t="n"/>
       <c r="I8" s="45" t="n"/>
       <c r="J8" s="45" t="n"/>
       <c r="K8" s="45" t="n"/>
       <c r="L8" s="45" t="n"/>
-      <c r="M8" s="61" t="n"/>
-      <c r="N8" s="61" t="n"/>
+      <c r="M8" s="58" t="n"/>
+      <c r="N8" s="58" t="n"/>
       <c r="O8" s="18" t="n"/>
       <c r="P8" s="18" t="n"/>
       <c r="Q8" s="18" t="n"/>
       <c r="R8" s="18" t="n"/>
       <c r="S8" s="18" t="n"/>
-      <c r="T8" s="62" t="n"/>
-      <c r="U8" s="62" t="n"/>
+      <c r="T8" s="59" t="n"/>
+      <c r="U8" s="59" t="n"/>
       <c r="V8" s="18" t="n"/>
       <c r="W8" s="18" t="n"/>
       <c r="X8" s="18" t="n"/>
       <c r="Y8" s="18" t="n"/>
       <c r="Z8" s="18" t="n"/>
-      <c r="AA8" s="60" t="n"/>
-      <c r="AB8" s="60" t="n"/>
+      <c r="AA8" s="57" t="n"/>
+      <c r="AB8" s="57" t="n"/>
       <c r="AC8" s="18" t="n"/>
       <c r="AD8" s="45" t="n"/>
       <c r="AE8" s="19" t="n"/>
@@ -1220,8 +1202,8 @@
       <c r="C9" s="46" t="n"/>
       <c r="D9" s="46" t="n"/>
       <c r="E9" s="46" t="n"/>
-      <c r="F9" s="56" t="n"/>
-      <c r="G9" s="56" t="n"/>
+      <c r="F9" s="55" t="n"/>
+      <c r="G9" s="55" t="n"/>
       <c r="H9" s="46" t="n"/>
       <c r="I9" s="46" t="n"/>
       <c r="J9" s="46" t="n"/>
@@ -1234,8 +1216,8 @@
       <c r="Q9" s="47" t="n"/>
       <c r="R9" s="47" t="n"/>
       <c r="S9" s="47" t="n"/>
-      <c r="T9" s="59" t="n"/>
-      <c r="U9" s="59" t="n"/>
+      <c r="T9" s="56" t="n"/>
+      <c r="U9" s="56" t="n"/>
       <c r="V9" s="46" t="n"/>
       <c r="W9" s="46" t="n"/>
       <c r="X9" s="46" t="n"/>
@@ -1260,29 +1242,29 @@
       <c r="C10" s="46" t="n"/>
       <c r="D10" s="18" t="n"/>
       <c r="E10" s="46" t="n"/>
-      <c r="F10" s="56" t="n"/>
-      <c r="G10" s="60" t="n"/>
+      <c r="F10" s="55" t="n"/>
+      <c r="G10" s="57" t="n"/>
       <c r="H10" s="46" t="n"/>
       <c r="I10" s="46" t="n"/>
       <c r="J10" s="18" t="n"/>
       <c r="K10" s="46" t="n"/>
       <c r="L10" s="46" t="n"/>
-      <c r="M10" s="60" t="n"/>
+      <c r="M10" s="57" t="n"/>
       <c r="N10" s="54" t="n"/>
       <c r="O10" s="47" t="n"/>
       <c r="P10" s="18" t="n"/>
       <c r="Q10" s="47" t="n"/>
       <c r="R10" s="47" t="n"/>
       <c r="S10" s="18" t="n"/>
-      <c r="T10" s="59" t="n"/>
-      <c r="U10" s="59" t="n"/>
+      <c r="T10" s="56" t="n"/>
+      <c r="U10" s="56" t="n"/>
       <c r="V10" s="18" t="n"/>
       <c r="W10" s="46" t="n"/>
       <c r="X10" s="46" t="n"/>
       <c r="Y10" s="46" t="n"/>
       <c r="Z10" s="46" t="n"/>
       <c r="AA10" s="54" t="n"/>
-      <c r="AB10" s="61" t="n"/>
+      <c r="AB10" s="58" t="n"/>
       <c r="AC10" s="45" t="n"/>
       <c r="AD10" s="18" t="n"/>
       <c r="AE10" s="39" t="n"/>
@@ -1300,22 +1282,22 @@
       <c r="C11" s="47" t="n"/>
       <c r="D11" s="47" t="n"/>
       <c r="E11" s="47" t="n"/>
-      <c r="F11" s="56" t="n"/>
-      <c r="G11" s="56" t="n"/>
+      <c r="F11" s="55" t="n"/>
+      <c r="G11" s="55" t="n"/>
       <c r="H11" s="46" t="n"/>
       <c r="I11" s="46" t="n"/>
       <c r="J11" s="46" t="n"/>
-      <c r="K11" s="63" t="n"/>
-      <c r="L11" s="63" t="n"/>
-      <c r="M11" s="64" t="n"/>
-      <c r="N11" s="64" t="n"/>
-      <c r="O11" s="63" t="n"/>
-      <c r="P11" s="63" t="n"/>
-      <c r="Q11" s="63" t="n"/>
+      <c r="K11" s="60" t="n"/>
+      <c r="L11" s="60" t="n"/>
+      <c r="M11" s="61" t="n"/>
+      <c r="N11" s="61" t="n"/>
+      <c r="O11" s="60" t="n"/>
+      <c r="P11" s="60" t="n"/>
+      <c r="Q11" s="60" t="n"/>
       <c r="R11" s="46" t="n"/>
       <c r="S11" s="46" t="n"/>
-      <c r="T11" s="59" t="n"/>
-      <c r="U11" s="59" t="n"/>
+      <c r="T11" s="56" t="n"/>
+      <c r="U11" s="56" t="n"/>
       <c r="V11" s="46" t="n"/>
       <c r="W11" s="46" t="n"/>
       <c r="X11" s="46" t="n"/>
@@ -1340,29 +1322,29 @@
       <c r="C12" s="46" t="n"/>
       <c r="D12" s="46" t="n"/>
       <c r="E12" s="18" t="n"/>
-      <c r="F12" s="60" t="n"/>
-      <c r="G12" s="56" t="n"/>
+      <c r="F12" s="57" t="n"/>
+      <c r="G12" s="55" t="n"/>
       <c r="H12" s="45" t="n"/>
       <c r="I12" s="45" t="n"/>
       <c r="J12" s="46" t="n"/>
       <c r="K12" s="45" t="n"/>
       <c r="L12" s="45" t="n"/>
       <c r="M12" s="54" t="n"/>
-      <c r="N12" s="61" t="n"/>
+      <c r="N12" s="58" t="n"/>
       <c r="O12" s="45" t="n"/>
       <c r="P12" s="46" t="n"/>
       <c r="Q12" s="45" t="n"/>
       <c r="R12" s="45" t="n"/>
       <c r="S12" s="46" t="n"/>
-      <c r="T12" s="61" t="n"/>
-      <c r="U12" s="61" t="n"/>
+      <c r="T12" s="58" t="n"/>
+      <c r="U12" s="58" t="n"/>
       <c r="V12" s="46" t="n"/>
       <c r="W12" s="45" t="n"/>
       <c r="X12" s="45" t="n"/>
       <c r="Y12" s="45" t="n"/>
       <c r="Z12" s="45" t="n"/>
-      <c r="AA12" s="61" t="n"/>
-      <c r="AB12" s="61" t="n"/>
+      <c r="AA12" s="58" t="n"/>
+      <c r="AB12" s="58" t="n"/>
       <c r="AC12" s="45" t="n"/>
       <c r="AD12" s="18" t="n"/>
       <c r="AE12" s="19" t="n"/>
@@ -1380,8 +1362,8 @@
       <c r="C13" s="47" t="n"/>
       <c r="D13" s="47" t="n"/>
       <c r="E13" s="47" t="n"/>
-      <c r="F13" s="56" t="n"/>
-      <c r="G13" s="56" t="n"/>
+      <c r="F13" s="55" t="n"/>
+      <c r="G13" s="55" t="n"/>
       <c r="H13" s="46" t="n"/>
       <c r="I13" s="46" t="n"/>
       <c r="J13" s="46" t="n"/>
@@ -1401,8 +1383,8 @@
       <c r="X13" s="18" t="n"/>
       <c r="Y13" s="18" t="n"/>
       <c r="Z13" s="18" t="n"/>
-      <c r="AA13" s="60" t="n"/>
-      <c r="AB13" s="60" t="n"/>
+      <c r="AA13" s="57" t="n"/>
+      <c r="AB13" s="57" t="n"/>
       <c r="AC13" s="18" t="n"/>
       <c r="AD13" s="46" t="n"/>
       <c r="AE13" s="19" t="n"/>
@@ -1420,8 +1402,8 @@
       <c r="C14" s="47" t="n"/>
       <c r="D14" s="47" t="n"/>
       <c r="E14" s="47" t="n"/>
-      <c r="F14" s="56" t="n"/>
-      <c r="G14" s="56" t="n"/>
+      <c r="F14" s="55" t="n"/>
+      <c r="G14" s="55" t="n"/>
       <c r="H14" s="46" t="n"/>
       <c r="I14" s="46" t="n"/>
       <c r="J14" s="46" t="n"/>
@@ -1441,8 +1423,8 @@
       <c r="X14" s="18" t="n"/>
       <c r="Y14" s="18" t="n"/>
       <c r="Z14" s="18" t="n"/>
-      <c r="AA14" s="60" t="n"/>
-      <c r="AB14" s="60" t="n"/>
+      <c r="AA14" s="57" t="n"/>
+      <c r="AB14" s="57" t="n"/>
       <c r="AC14" s="18" t="n"/>
       <c r="AD14" s="46" t="n"/>
       <c r="AE14" s="19" t="n"/>
@@ -1456,33 +1438,33 @@
           <t>PRO ROSAS FERNANDEZ RODRIGO</t>
         </is>
       </c>
-      <c r="B15" s="65" t="n"/>
-      <c r="C15" s="65" t="n"/>
-      <c r="D15" s="55" t="n"/>
-      <c r="E15" s="65" t="n"/>
-      <c r="F15" s="65" t="n"/>
-      <c r="G15" s="55" t="n"/>
+      <c r="B15" s="62" t="n"/>
+      <c r="C15" s="62" t="n"/>
+      <c r="D15" s="63" t="n"/>
+      <c r="E15" s="62" t="n"/>
+      <c r="F15" s="62" t="n"/>
+      <c r="G15" s="63" t="n"/>
       <c r="H15" s="45" t="n"/>
       <c r="I15" s="45" t="n"/>
       <c r="J15" s="46" t="n"/>
       <c r="K15" s="45" t="n"/>
       <c r="L15" s="45" t="n"/>
       <c r="M15" s="54" t="n"/>
-      <c r="N15" s="61" t="n"/>
+      <c r="N15" s="58" t="n"/>
       <c r="O15" s="45" t="n"/>
       <c r="P15" s="46" t="n"/>
       <c r="Q15" s="45" t="n"/>
       <c r="R15" s="45" t="n"/>
       <c r="S15" s="46" t="n"/>
-      <c r="T15" s="61" t="n"/>
-      <c r="U15" s="61" t="n"/>
+      <c r="T15" s="58" t="n"/>
+      <c r="U15" s="58" t="n"/>
       <c r="V15" s="47" t="n"/>
       <c r="W15" s="18" t="n"/>
       <c r="X15" s="18" t="n"/>
       <c r="Y15" s="18" t="n"/>
       <c r="Z15" s="18" t="n"/>
-      <c r="AA15" s="60" t="n"/>
-      <c r="AB15" s="60" t="n"/>
+      <c r="AA15" s="57" t="n"/>
+      <c r="AB15" s="57" t="n"/>
       <c r="AC15" s="18" t="n"/>
       <c r="AD15" s="46" t="n"/>
       <c r="AE15" s="19" t="n"/>
@@ -1500,37 +1482,29 @@
       <c r="C16" s="18" t="n"/>
       <c r="D16" s="47" t="n"/>
       <c r="E16" s="18" t="n"/>
-      <c r="F16" s="60" t="n"/>
-      <c r="G16" s="56" t="n"/>
-      <c r="H16" s="45" t="n"/>
-      <c r="I16" s="66" t="inlineStr">
-        <is>
-          <t>DA</t>
-        </is>
-      </c>
-      <c r="J16" s="66" t="inlineStr">
-        <is>
-          <t>DA</t>
-        </is>
-      </c>
-      <c r="K16" s="45" t="n"/>
-      <c r="L16" s="45" t="n"/>
-      <c r="M16" s="54" t="n"/>
-      <c r="N16" s="60" t="n"/>
+      <c r="F16" s="57" t="n"/>
+      <c r="G16" s="55" t="n"/>
+      <c r="H16" s="64" t="n"/>
+      <c r="I16" s="64" t="n"/>
+      <c r="J16" s="65" t="n"/>
+      <c r="K16" s="64" t="n"/>
+      <c r="L16" s="64" t="n"/>
+      <c r="M16" s="65" t="n"/>
+      <c r="N16" s="62" t="n"/>
       <c r="O16" s="18" t="n"/>
       <c r="P16" s="46" t="n"/>
       <c r="Q16" s="18" t="n"/>
       <c r="R16" s="18" t="n"/>
       <c r="S16" s="46" t="n"/>
-      <c r="T16" s="60" t="n"/>
-      <c r="U16" s="60" t="n"/>
+      <c r="T16" s="57" t="n"/>
+      <c r="U16" s="57" t="n"/>
       <c r="V16" s="46" t="n"/>
       <c r="W16" s="18" t="n"/>
       <c r="X16" s="18" t="n"/>
       <c r="Y16" s="18" t="n"/>
       <c r="Z16" s="18" t="n"/>
-      <c r="AA16" s="60" t="n"/>
-      <c r="AB16" s="60" t="n"/>
+      <c r="AA16" s="57" t="n"/>
+      <c r="AB16" s="57" t="n"/>
       <c r="AC16" s="18" t="n"/>
       <c r="AD16" s="46" t="n"/>
       <c r="AE16" s="19" t="n"/>
@@ -1548,15 +1522,15 @@
       <c r="C17" s="47" t="n"/>
       <c r="D17" s="47" t="n"/>
       <c r="E17" s="47" t="n"/>
-      <c r="F17" s="56" t="n"/>
-      <c r="G17" s="56" t="n"/>
-      <c r="H17" s="57" t="n"/>
-      <c r="I17" s="57" t="n"/>
-      <c r="J17" s="57" t="n"/>
-      <c r="K17" s="57" t="n"/>
-      <c r="L17" s="57" t="n"/>
-      <c r="M17" s="57" t="n"/>
-      <c r="N17" s="57" t="n"/>
+      <c r="F17" s="55" t="n"/>
+      <c r="G17" s="55" t="n"/>
+      <c r="H17" s="46" t="n"/>
+      <c r="I17" s="46" t="n"/>
+      <c r="J17" s="46" t="n"/>
+      <c r="K17" s="46" t="n"/>
+      <c r="L17" s="46" t="n"/>
+      <c r="M17" s="54" t="n"/>
+      <c r="N17" s="54" t="n"/>
       <c r="O17" s="46" t="n"/>
       <c r="P17" s="46" t="n"/>
       <c r="Q17" s="46" t="n"/>
@@ -1564,13 +1538,13 @@
       <c r="S17" s="46" t="n"/>
       <c r="T17" s="54" t="n"/>
       <c r="U17" s="54" t="n"/>
-      <c r="V17" s="46" t="n"/>
-      <c r="W17" s="46" t="n"/>
-      <c r="X17" s="46" t="n"/>
-      <c r="Y17" s="46" t="n"/>
-      <c r="Z17" s="46" t="n"/>
-      <c r="AA17" s="54" t="n"/>
-      <c r="AB17" s="54" t="n"/>
+      <c r="V17" s="65" t="n"/>
+      <c r="W17" s="65" t="n"/>
+      <c r="X17" s="65" t="n"/>
+      <c r="Y17" s="65" t="n"/>
+      <c r="Z17" s="65" t="n"/>
+      <c r="AA17" s="65" t="n"/>
+      <c r="AB17" s="65" t="n"/>
       <c r="AC17" s="46" t="n"/>
       <c r="AD17" s="46" t="n"/>
       <c r="AE17" s="19" t="n"/>
@@ -1597,13 +1571,13 @@
       <c r="L18" s="46" t="n"/>
       <c r="M18" s="54" t="n"/>
       <c r="N18" s="54" t="n"/>
-      <c r="O18" s="57" t="n"/>
-      <c r="P18" s="57" t="n"/>
-      <c r="Q18" s="57" t="n"/>
-      <c r="R18" s="57" t="n"/>
-      <c r="S18" s="57" t="n"/>
-      <c r="T18" s="57" t="n"/>
-      <c r="U18" s="57" t="n"/>
+      <c r="O18" s="65" t="n"/>
+      <c r="P18" s="65" t="n"/>
+      <c r="Q18" s="65" t="n"/>
+      <c r="R18" s="65" t="n"/>
+      <c r="S18" s="65" t="n"/>
+      <c r="T18" s="65" t="n"/>
+      <c r="U18" s="65" t="n"/>
       <c r="V18" s="46" t="n"/>
       <c r="W18" s="46" t="n"/>
       <c r="X18" s="46" t="n"/>
@@ -1635,8 +1609,8 @@
       <c r="J19" s="47" t="n"/>
       <c r="K19" s="47" t="n"/>
       <c r="L19" s="47" t="n"/>
-      <c r="M19" s="56" t="n"/>
-      <c r="N19" s="56" t="n"/>
+      <c r="M19" s="55" t="n"/>
+      <c r="N19" s="55" t="n"/>
       <c r="O19" s="46" t="n"/>
       <c r="P19" s="46" t="n"/>
       <c r="Q19" s="46" t="n"/>
@@ -1645,27 +1619,15 @@
       <c r="T19" s="54" t="n"/>
       <c r="U19" s="54" t="n"/>
       <c r="V19" s="46" t="n"/>
-      <c r="W19" s="67" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
-      <c r="X19" s="67" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
-      <c r="Y19" s="67" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
+      <c r="W19" s="46" t="n"/>
+      <c r="X19" s="46" t="n"/>
+      <c r="Y19" s="46" t="n"/>
       <c r="Z19" s="46" t="n"/>
       <c r="AA19" s="54" t="n"/>
       <c r="AB19" s="54" t="n"/>
-      <c r="AC19" s="46" t="n"/>
-      <c r="AD19" s="18" t="n"/>
-      <c r="AE19" s="19" t="n"/>
+      <c r="AC19" s="65" t="n"/>
+      <c r="AD19" s="62" t="n"/>
+      <c r="AE19" s="66" t="n"/>
       <c r="AF19" s="19" t="n"/>
       <c r="AG19" s="19" t="n"/>
       <c r="AH19" s="19" t="n"/>

</xml_diff>